<commit_message>
cambios en el modelado mecanico para ingreso de la placa
</commit_message>
<xml_diff>
--- a/listaDeMatertiales.xlsx
+++ b/listaDeMatertiales.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\universidad\tesis\materialescomprados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\universidad\tesis\simulador_de_Extraccion_de_polipos_intestinales\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="5070"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="5070" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
   <si>
     <t>Materiales</t>
   </si>
@@ -123,13 +124,82 @@
   </si>
   <si>
     <t>total bs.</t>
+  </si>
+  <si>
+    <t>Raspberry Pi 4</t>
+  </si>
+  <si>
+    <t>Fuente de alimentación oficial para Raspberry Pi 4 (USB-C 5V 3A)</t>
+  </si>
+  <si>
+    <t>Módulo de Procesamiento y Gráficos</t>
+  </si>
+  <si>
+    <t>Placa de Desarrollo STM32 Nucleo-32:</t>
+  </si>
+  <si>
+    <t>Cable USB a Micro-USB</t>
+  </si>
+  <si>
+    <t>adaptador Micro-HDMI a HDMI</t>
+  </si>
+  <si>
+    <t>Tiras de Espadines Hembra</t>
+  </si>
+  <si>
+    <t>bornera conectores por tornillo</t>
+  </si>
+  <si>
+    <t>Transistores TIP120</t>
+  </si>
+  <si>
+    <t>Diodos Rectificadores 1N4007</t>
+  </si>
+  <si>
+    <t>Resistencias de 4.7kΩ</t>
+  </si>
+  <si>
+    <t>Resistencias de 10kΩ</t>
+  </si>
+  <si>
+    <t>Resistencias de 1kΩ</t>
+  </si>
+  <si>
+    <t>Resistencias de 220Ω</t>
+  </si>
+  <si>
+    <t>botones autorretorno con tuerca</t>
+  </si>
+  <si>
+    <t>Módulo Sensorial y Háptico</t>
+  </si>
+  <si>
+    <t>Sensor Magnético I2C AS5600</t>
+  </si>
+  <si>
+    <t>Motores Vibradores (Micro-motores tipo moneda)</t>
+  </si>
+  <si>
+    <t>Tubo flexible TPU / manguera</t>
+  </si>
+  <si>
+    <t>ventilador 5v</t>
+  </si>
+  <si>
+    <t>MicroSD (Mínimo 32GB)</t>
+  </si>
+  <si>
+    <t>LED RGB catodo comun</t>
+  </si>
+  <si>
+    <t>Encoders Rotatorios Modulares HW-040</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,16 +232,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -194,11 +279,82 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -218,6 +374,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -227,7 +384,61 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -518,10 +729,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="9"/>
+      <c r="D3" s="10"/>
       <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
@@ -530,10 +741,10 @@
       </c>
     </row>
     <row r="4" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C4" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="10"/>
+      <c r="C4" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
@@ -680,7 +891,7 @@
       <c r="D14" s="3">
         <v>1</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="9">
         <v>67.5</v>
       </c>
       <c r="F14" s="2">
@@ -749,10 +960,10 @@
       </c>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="11"/>
+      <c r="D19" s="12"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
@@ -908,4 +1119,468 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B3:E35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="60" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="28"/>
+      <c r="D4" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="26"/>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="20">
+        <v>1</v>
+      </c>
+      <c r="D6" s="14">
+        <v>1500</v>
+      </c>
+      <c r="E6" s="14">
+        <f>C6*D6</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="15">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>18</v>
+      </c>
+      <c r="E7" s="2">
+        <f>C7*D7</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="15">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>185</v>
+      </c>
+      <c r="E8" s="2">
+        <f t="shared" ref="E8:E23" si="0">C8*D8</f>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="15">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2">
+        <v>62.5</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="0"/>
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="15">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>140</v>
+      </c>
+      <c r="E10" s="2">
+        <f t="shared" si="0"/>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="15">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2">
+        <v>52</v>
+      </c>
+      <c r="E11" s="2">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="18">
+        <v>1</v>
+      </c>
+      <c r="D12" s="13">
+        <v>45</v>
+      </c>
+      <c r="E12" s="13">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="26"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="20">
+        <v>1</v>
+      </c>
+      <c r="D14" s="14">
+        <v>4</v>
+      </c>
+      <c r="E14" s="14">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="15">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="15">
+        <v>2</v>
+      </c>
+      <c r="D16" s="2">
+        <v>3</v>
+      </c>
+      <c r="E16" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="15">
+        <v>2</v>
+      </c>
+      <c r="D17" s="9">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="15">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="15">
+        <v>5</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="15">
+        <v>2</v>
+      </c>
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="15">
+        <v>3</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="15">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="18">
+        <v>4</v>
+      </c>
+      <c r="D23" s="13">
+        <v>5</v>
+      </c>
+      <c r="E23" s="13">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="32" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="33"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="26"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="20">
+        <v>2</v>
+      </c>
+      <c r="D25" s="14">
+        <v>25</v>
+      </c>
+      <c r="E25" s="14">
+        <f>C25*D25</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="15">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2">
+        <v>20</v>
+      </c>
+      <c r="E26" s="2">
+        <f t="shared" ref="E26:E27" si="1">C26*D26</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="18">
+        <v>2</v>
+      </c>
+      <c r="D27" s="13">
+        <v>5</v>
+      </c>
+      <c r="E27" s="13">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="33"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="26"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="14">
+        <v>1</v>
+      </c>
+      <c r="E29" s="14">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="15">
+        <v>10</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2">
+        <f>D31</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="15">
+        <v>10</v>
+      </c>
+      <c r="D32" s="2">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2">
+        <f t="shared" ref="E32" si="2">D32</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2">
+        <f t="shared" ref="E33" si="3">D33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34" s="15">
+        <v>4</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2">
+        <f t="shared" ref="E34" si="4">C34*D34</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="2"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="2">
+        <f>SUM(E6:E34)</f>
+        <v>2584.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B28:C28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
cambios para la prueba v1
</commit_message>
<xml_diff>
--- a/listaDeMatertiales.xlsx
+++ b/listaDeMatertiales.xlsx
@@ -375,15 +375,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -410,34 +401,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -729,10 +729,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="10"/>
+      <c r="D3" s="25"/>
       <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
@@ -741,10 +741,10 @@
       </c>
     </row>
     <row r="4" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C4" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="11"/>
+      <c r="C4" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="26"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
@@ -960,10 +960,10 @@
       </c>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="12"/>
+      <c r="D19" s="27"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
@@ -1134,45 +1134,45 @@
   <sheetData>
     <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="28"/>
-      <c r="D4" s="29" t="s">
+      <c r="C4" s="33"/>
+      <c r="D4" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="23" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="26"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="21"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="20">
-        <v>1</v>
-      </c>
-      <c r="D6" s="14">
+      <c r="C6" s="17">
+        <v>1</v>
+      </c>
+      <c r="D6" s="11">
         <v>1500</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="11">
         <f>C6*D6</f>
         <v>1500</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="12">
         <v>1</v>
       </c>
       <c r="D7" s="2">
@@ -1184,10 +1184,10 @@
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="12">
         <v>1</v>
       </c>
       <c r="D8" s="2">
@@ -1202,7 +1202,7 @@
       <c r="B9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="12">
         <v>1</v>
       </c>
       <c r="D9" s="2">
@@ -1217,7 +1217,7 @@
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="12">
         <v>1</v>
       </c>
       <c r="D10" s="2">
@@ -1232,7 +1232,7 @@
       <c r="B11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="12">
         <v>1</v>
       </c>
       <c r="D11" s="2">
@@ -1244,48 +1244,48 @@
       </c>
     </row>
     <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="18">
-        <v>1</v>
-      </c>
-      <c r="D12" s="13">
+      <c r="C12" s="15">
+        <v>1</v>
+      </c>
+      <c r="D12" s="10">
         <v>45</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="10">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="26"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="20">
-        <v>1</v>
-      </c>
-      <c r="D14" s="14">
+      <c r="C14" s="17">
+        <v>1</v>
+      </c>
+      <c r="D14" s="11">
         <v>4</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="11">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="12">
         <v>2</v>
       </c>
       <c r="D15" s="2">
@@ -1300,7 +1300,7 @@
       <c r="B16" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="12">
         <v>2</v>
       </c>
       <c r="D16" s="2">
@@ -1315,7 +1315,7 @@
       <c r="B17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="12">
         <v>2</v>
       </c>
       <c r="D17" s="9">
@@ -1330,7 +1330,7 @@
       <c r="B18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="12">
         <v>4</v>
       </c>
       <c r="D18" s="2">
@@ -1345,7 +1345,7 @@
       <c r="B19" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="12">
         <v>5</v>
       </c>
       <c r="D19" s="2">
@@ -1360,7 +1360,7 @@
       <c r="B20" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="12">
         <v>2</v>
       </c>
       <c r="D20" s="2">
@@ -1375,7 +1375,7 @@
       <c r="B21" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="15">
+      <c r="C21" s="12">
         <v>3</v>
       </c>
       <c r="D21" s="2">
@@ -1390,7 +1390,7 @@
       <c r="B22" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="12">
         <v>1</v>
       </c>
       <c r="D22" s="2">
@@ -1402,39 +1402,39 @@
       </c>
     </row>
     <row r="23" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="15">
         <v>4</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="10">
         <v>5</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="10">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="26"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="21"/>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="20">
-        <v>2</v>
-      </c>
-      <c r="D25" s="14">
+      <c r="C25" s="17">
+        <v>2</v>
+      </c>
+      <c r="D25" s="11">
         <v>25</v>
       </c>
-      <c r="E25" s="14">
+      <c r="E25" s="11">
         <f>C25*D25</f>
         <v>50</v>
       </c>
@@ -1443,7 +1443,7 @@
       <c r="B26" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C26" s="12">
         <v>2</v>
       </c>
       <c r="D26" s="2">
@@ -1455,47 +1455,47 @@
       </c>
     </row>
     <row r="27" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="18">
-        <v>2</v>
-      </c>
-      <c r="D27" s="13">
+      <c r="C27" s="15">
+        <v>2</v>
+      </c>
+      <c r="D27" s="10">
         <v>5</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="10">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="33"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="26"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="21"/>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="14">
-        <v>1</v>
-      </c>
-      <c r="E29" s="14">
+      <c r="D29" s="11">
+        <v>1</v>
+      </c>
+      <c r="E29" s="11">
         <v>206</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="12" t="s">
         <v>13</v>
       </c>
       <c r="D30" s="2">
@@ -1506,10 +1506,10 @@
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="12">
         <v>10</v>
       </c>
       <c r="D31" s="2">
@@ -1521,10 +1521,10 @@
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="12">
         <v>10</v>
       </c>
       <c r="D32" s="2">
@@ -1536,10 +1536,10 @@
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="12" t="s">
         <v>27</v>
       </c>
       <c r="D33" s="2"/>
@@ -1549,10 +1549,10 @@
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="15">
+      <c r="C34" s="12">
         <v>4</v>
       </c>
       <c r="D34" s="2"/>
@@ -1563,7 +1563,7 @@
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
-      <c r="C35" s="31"/>
+      <c r="C35" s="24"/>
       <c r="D35" s="5" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Actualizar la escena de Unity, los prefabs y los textos del tutorial para su uso en diferentes pantallas..
Aplicar varias actualizaciones al proyecto Unity: reemplazar los binarios y recursos de datos compilados/administrados para la compilación de Windows, ajustar los anclajes/posiciones/tamaños de UI RectTransform en EscenaGameplay.unity, cambiar la alineación del texto del prefab Molde_BotonArchivo y refinar el texto del tutorial/instrucciones en español para mayor claridad y coherencia. También agregar referencias de UI (succion/limpiado) e incluir una hoja de cálculo de materiales actualizada (listaDeMatertiales.xlsx). Estos cambios parecen ser ajustes de diseño y contenido para la escena de juego y los recursos relacionados.
</commit_message>
<xml_diff>
--- a/listaDeMatertiales.xlsx
+++ b/listaDeMatertiales.xlsx
@@ -9,11 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="5070" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="5070" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="131">
   <si>
     <t>Materiales</t>
   </si>
@@ -126,12 +127,6 @@
     <t>total bs.</t>
   </si>
   <si>
-    <t>Raspberry Pi 4</t>
-  </si>
-  <si>
-    <t>Fuente de alimentación oficial para Raspberry Pi 4 (USB-C 5V 3A)</t>
-  </si>
-  <si>
     <t>Módulo de Procesamiento y Gráficos</t>
   </si>
   <si>
@@ -141,15 +136,9 @@
     <t>Cable USB a Micro-USB</t>
   </si>
   <si>
-    <t>adaptador Micro-HDMI a HDMI</t>
-  </si>
-  <si>
     <t>Tiras de Espadines Hembra</t>
   </si>
   <si>
-    <t>bornera conectores por tornillo</t>
-  </si>
-  <si>
     <t>Transistores TIP120</t>
   </si>
   <si>
@@ -162,12 +151,6 @@
     <t>Resistencias de 10kΩ</t>
   </si>
   <si>
-    <t>Resistencias de 1kΩ</t>
-  </si>
-  <si>
-    <t>Resistencias de 220Ω</t>
-  </si>
-  <si>
     <t>botones autorretorno con tuerca</t>
   </si>
   <si>
@@ -180,19 +163,262 @@
     <t>Motores Vibradores (Micro-motores tipo moneda)</t>
   </si>
   <si>
+    <t>Encoders Rotatorios Modulares HW-040</t>
+  </si>
+  <si>
+    <t>bornera conectores por tornillo de 2</t>
+  </si>
+  <si>
+    <t>capacitor ceramico de 10 nf</t>
+  </si>
+  <si>
+    <t>PLA(experimental como produccion)kg</t>
+  </si>
+  <si>
+    <t>tiempo de uso en una impresora 3d (propia) horas</t>
+  </si>
+  <si>
+    <t>tira de goma 1/4 demetro</t>
+  </si>
+  <si>
+    <t>cable de telefono ( metros)</t>
+  </si>
+  <si>
+    <t>cable lan (metros)</t>
+  </si>
+  <si>
+    <t>barras de psilicona</t>
+  </si>
+  <si>
+    <t>Tubo flexible TPU / manguera (metros)</t>
+  </si>
+  <si>
+    <t>creacion de pcb por cnc (costo de todas las placas)</t>
+  </si>
+  <si>
+    <t>medios exernos usados</t>
+  </si>
+  <si>
+    <t>diseño del circuito (dias)</t>
+  </si>
+  <si>
+    <t>diseño mecanico solidworks (dias)</t>
+  </si>
+  <si>
+    <t>programacion del programa en unity</t>
+  </si>
+  <si>
+    <t>programacion del circuito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pruebas de funcionamiento </t>
+  </si>
+  <si>
+    <t>elementos electronicos o insumos electronicos</t>
+  </si>
+  <si>
+    <t>trabajo  propio con las faces de experimentacion</t>
+  </si>
+  <si>
+    <t>soldadura por horas (con materia prima)</t>
+  </si>
+  <si>
+    <t>Tornillos M3/M4 (por lote)</t>
+  </si>
+  <si>
+    <t>Tuercas insertables M3/M4 (por lote)</t>
+  </si>
+  <si>
+    <t>M+B4:E40ateriales</t>
+  </si>
+  <si>
+    <t>Componente</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Costo unitario (Bs.)</t>
+  </si>
+  <si>
+    <t>Subtotal (Bs.)</t>
+  </si>
+  <si>
+    <t>Placa STM32 Nucleo-32</t>
+  </si>
+  <si>
+    <t>Tiras de espadines hembra</t>
+  </si>
+  <si>
+    <t>Borneras conectoras por tornillo</t>
+  </si>
+  <si>
+    <t>Diodos rectificadores 1N4007</t>
+  </si>
+  <si>
+    <t>Resistencias de 4.7 kΩ</t>
+  </si>
+  <si>
+    <t>Resistencias de 10 kΩ</t>
+  </si>
+  <si>
+    <t>Capacitores cerámicos de 10 nF</t>
+  </si>
+  <si>
+    <t>Cable telefónico</t>
+  </si>
+  <si>
+    <t>2 m</t>
+  </si>
+  <si>
+    <t>Cable LAN</t>
+  </si>
+  <si>
+    <t>Botones autorretorno con tuerca</t>
+  </si>
+  <si>
+    <t>Total materiales electrónicos</t>
+  </si>
+  <si>
+    <t>369 Bs.</t>
+  </si>
+  <si>
+    <t>Sensor magnético I2C AS5600</t>
+  </si>
+  <si>
+    <t>Encoders rotatorios modulares HW-040</t>
+  </si>
+  <si>
+    <t>Motores vibradores tipo moneda</t>
+  </si>
+  <si>
+    <t>Total módulo sensorial y háptico</t>
+  </si>
+  <si>
+    <t>80 Bs.</t>
+  </si>
+  <si>
+    <t>PLA para impresión 3D</t>
+  </si>
+  <si>
+    <t>3 kg</t>
+  </si>
+  <si>
+    <t>Tiempo de impresión 3D</t>
+  </si>
+  <si>
+    <t>105 h</t>
+  </si>
+  <si>
+    <t>Tuercas insertables M3/M4</t>
+  </si>
+  <si>
     <t>Tubo flexible TPU / manguera</t>
   </si>
   <si>
-    <t>ventilador 5v</t>
-  </si>
-  <si>
-    <t>MicroSD (Mínimo 32GB)</t>
-  </si>
-  <si>
-    <t>LED RGB catodo comun</t>
-  </si>
-  <si>
-    <t>Encoders Rotatorios Modulares HW-040</t>
+    <t>3 m</t>
+  </si>
+  <si>
+    <t>Barras de silicona</t>
+  </si>
+  <si>
+    <t>Tira de goma 1/4 de metro</t>
+  </si>
+  <si>
+    <t>Total materiales mecánicos y fabricación</t>
+  </si>
+  <si>
+    <t>2158 Bs.</t>
+  </si>
+  <si>
+    <t>Concepto</t>
+  </si>
+  <si>
+    <t>Fabricación de PCB por CNC</t>
+  </si>
+  <si>
+    <t>Total fabricación externa</t>
+  </si>
+  <si>
+    <t>150 Bs.</t>
+  </si>
+  <si>
+    <t>Actividad</t>
+  </si>
+  <si>
+    <t>Diseño del circuito</t>
+  </si>
+  <si>
+    <t>18 días</t>
+  </si>
+  <si>
+    <t>Diseño mecánico en SolidWorks</t>
+  </si>
+  <si>
+    <t>34 días</t>
+  </si>
+  <si>
+    <t>Programación del circuito</t>
+  </si>
+  <si>
+    <t>12 días</t>
+  </si>
+  <si>
+    <t>Programación en Unity</t>
+  </si>
+  <si>
+    <t>44 días</t>
+  </si>
+  <si>
+    <t>Pruebas de funcionamiento</t>
+  </si>
+  <si>
+    <t>7 días</t>
+  </si>
+  <si>
+    <t>Soldadura y ensamblaje</t>
+  </si>
+  <si>
+    <t>Total mano de obra y desarrollo</t>
+  </si>
+  <si>
+    <t>Cantidad          (12h x dia)</t>
+  </si>
+  <si>
+    <t>Costo unitario  (20Bs. x 1h)</t>
+  </si>
+  <si>
+    <t>Categoría</t>
+  </si>
+  <si>
+    <t>Total (Bs.)</t>
+  </si>
+  <si>
+    <t>Materiales electrónicos</t>
+  </si>
+  <si>
+    <t>Módulo sensorial y háptico</t>
+  </si>
+  <si>
+    <t>Materiales mecánicos y fabricación</t>
+  </si>
+  <si>
+    <t>Fabricación externa</t>
+  </si>
+  <si>
+    <t>Mano de obra y desarrollo</t>
+  </si>
+  <si>
+    <t>Costo total del prototipo</t>
+  </si>
+  <si>
+    <t>4 horas</t>
+  </si>
+  <si>
+    <t>27680 Bs.</t>
+  </si>
+  <si>
+    <t>30437 Bs.</t>
   </si>
 </sst>
 </file>
@@ -256,7 +482,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -350,11 +576,126 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -384,22 +725,13 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
@@ -412,6 +744,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -438,6 +773,69 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -729,10 +1127,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="25"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
@@ -741,10 +1139,10 @@
       </c>
     </row>
     <row r="4" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C4" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="26"/>
+      <c r="C4" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="24"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
@@ -960,10 +1358,10 @@
       </c>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="27"/>
+      <c r="D19" s="25"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
@@ -1123,10 +1521,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:E35"/>
+  <dimension ref="B3:E40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="60" customWidth="1"/>
+    <col min="2" max="2" width="72.140625" customWidth="1"/>
     <col min="3" max="3" width="16.28515625" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" customWidth="1"/>
     <col min="5" max="5" width="16.140625" customWidth="1"/>
@@ -1134,98 +1532,93 @@
   <sheetData>
     <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="18"/>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="12">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2">
+        <v>220</v>
+      </c>
+      <c r="E6" s="2">
+        <f t="shared" ref="E6:E18" si="0">C6*D6</f>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="12">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>52</v>
+      </c>
+      <c r="E7" s="2">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="18">
         <v>0</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="21"/>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="17">
-        <v>1</v>
-      </c>
-      <c r="D6" s="11">
-        <v>1500</v>
-      </c>
-      <c r="E6" s="11">
-        <f>C6*D6</f>
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="12">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2">
-        <v>18</v>
-      </c>
-      <c r="E7" s="2">
-        <f>C7*D7</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="12">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2">
-        <v>185</v>
-      </c>
-      <c r="E8" s="2">
-        <f t="shared" ref="E8:E23" si="0">C8*D8</f>
-        <v>185</v>
-      </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="12">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2">
-        <v>62.5</v>
-      </c>
-      <c r="E9" s="2">
+      <c r="B9" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="15">
+        <v>2</v>
+      </c>
+      <c r="D9" s="11">
+        <v>4</v>
+      </c>
+      <c r="E9" s="11">
         <f t="shared" si="0"/>
-        <v>62.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="2" t="s">
-        <v>36</v>
+      <c r="B10" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="C10" s="12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2">
-        <v>140</v>
+        <v>2</v>
       </c>
       <c r="E10" s="2">
         <f t="shared" si="0"/>
-        <v>140</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
@@ -1233,57 +1626,64 @@
         <v>37</v>
       </c>
       <c r="C11" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="2">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="E11" s="2">
         <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="15">
-        <v>1</v>
-      </c>
-      <c r="D12" s="10">
-        <v>45</v>
-      </c>
-      <c r="E12" s="10">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="17">
-        <v>1</v>
-      </c>
-      <c r="D14" s="11">
-        <v>4</v>
-      </c>
-      <c r="E14" s="11">
+      <c r="C12" s="12">
+        <v>2</v>
+      </c>
+      <c r="D12" s="9">
+        <v>2</v>
+      </c>
+      <c r="E12" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="12">
+        <v>4</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="12">
+        <v>8</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="13" t="s">
-        <v>40</v>
+      <c r="B15" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="C15" s="12">
         <v>2</v>
@@ -1298,289 +1698,978 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C16" s="12">
         <v>2</v>
       </c>
       <c r="D16" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E16" s="2">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C17" s="12">
         <v>2</v>
       </c>
-      <c r="D17" s="9">
-        <v>1</v>
+      <c r="D17" s="2">
+        <v>10</v>
       </c>
       <c r="E17" s="2">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="14">
+        <v>5</v>
+      </c>
+      <c r="D18" s="10">
+        <v>5</v>
+      </c>
+      <c r="E18" s="10">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="29"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="12">
-        <v>4</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1</v>
-      </c>
-      <c r="E18" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="12">
-        <v>5</v>
-      </c>
-      <c r="D19" s="2">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="12">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2">
-        <v>1</v>
-      </c>
-      <c r="E20" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
+      <c r="C20" s="15">
+        <v>2</v>
+      </c>
+      <c r="D20" s="11">
+        <v>25</v>
+      </c>
+      <c r="E20" s="11">
+        <f>C20*D20</f>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C21" s="12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" s="2">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E21" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="12">
-        <v>1</v>
-      </c>
-      <c r="D22" s="2">
-        <v>1</v>
+        <f t="shared" ref="E21:E22" si="1">C21*D21</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="14">
+        <v>2</v>
+      </c>
+      <c r="D22" s="10">
+        <v>5</v>
       </c>
       <c r="E22" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C23" s="15">
-        <v>4</v>
-      </c>
-      <c r="D23" s="10">
-        <v>5</v>
-      </c>
-      <c r="E23" s="10">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="C24" s="31"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="21"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" s="17">
-        <v>2</v>
-      </c>
-      <c r="D25" s="11">
-        <v>25</v>
-      </c>
-      <c r="E25" s="11">
-        <f>C25*D25</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B26" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="12">
-        <v>2</v>
-      </c>
-      <c r="D26" s="2">
-        <v>20</v>
-      </c>
-      <c r="E26" s="2">
-        <f t="shared" ref="E26:E27" si="1">C26*D26</f>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="15">
-        <v>2</v>
-      </c>
-      <c r="D27" s="10">
-        <v>5</v>
-      </c>
-      <c r="E27" s="10">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="30" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="21"/>
+    <row r="23" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="27"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="12">
+        <v>3</v>
+      </c>
+      <c r="D24" s="2">
+        <v>223</v>
+      </c>
+      <c r="E24" s="2">
+        <f>C24*D24</f>
+        <v>669</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="12">
+        <v>105</v>
+      </c>
+      <c r="D25" s="2">
+        <v>12</v>
+      </c>
+      <c r="E25" s="2">
+        <f>C25*D25</f>
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="22">
+        <v>1</v>
+      </c>
+      <c r="D26" s="2">
+        <v>60</v>
+      </c>
+      <c r="E26" s="2">
+        <f t="shared" ref="E26:E32" si="2">C26*D26</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="22">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2">
+        <v>60</v>
+      </c>
+      <c r="E27" s="2">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="12">
+        <v>3</v>
+      </c>
+      <c r="D28" s="2">
+        <v>20</v>
+      </c>
+      <c r="E28" s="2">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="12">
+        <v>2</v>
+      </c>
+      <c r="D29" s="2">
+        <v>2</v>
+      </c>
+      <c r="E29" s="2">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C30" s="12">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2">
+        <v>45</v>
+      </c>
+      <c r="E30" s="2">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="27"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="12">
+        <v>1</v>
+      </c>
+      <c r="D32" s="2">
+        <v>150</v>
+      </c>
+      <c r="E32" s="2">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="27"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="22">
+        <v>18</v>
+      </c>
+      <c r="D34" s="2">
+        <f>12*20</f>
+        <v>240</v>
+      </c>
+      <c r="E34" s="2">
+        <f>D34*C34</f>
+        <v>4320</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" s="22">
+        <v>34</v>
+      </c>
+      <c r="D35" s="2">
+        <f t="shared" ref="D35:D39" si="3">12*20</f>
+        <v>240</v>
+      </c>
+      <c r="E35" s="2">
+        <f t="shared" ref="E35:E39" si="4">D35*C35</f>
+        <v>8160</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="22">
         <v>12</v>
       </c>
-      <c r="C29" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="11">
-        <v>1</v>
-      </c>
-      <c r="E29" s="11">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="2">
-        <v>1</v>
-      </c>
-      <c r="E30" s="2">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="12">
-        <v>10</v>
-      </c>
-      <c r="D31" s="2">
-        <v>1</v>
-      </c>
-      <c r="E31" s="2">
-        <f>D31</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="12">
-        <v>10</v>
-      </c>
-      <c r="D32" s="2">
-        <v>1</v>
-      </c>
-      <c r="E32" s="2">
-        <f t="shared" ref="E32" si="2">D32</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2">
-        <f t="shared" ref="E33" si="3">D33</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C34" s="12">
-        <v>4</v>
-      </c>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2">
-        <f t="shared" ref="E34" si="4">C34*D34</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="2"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="5" t="s">
+      <c r="D36" s="2">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+      <c r="E36" s="2">
+        <f t="shared" si="4"/>
+        <v>2880</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B37" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" s="22">
+        <v>44</v>
+      </c>
+      <c r="D37" s="2">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+      <c r="E37" s="2">
+        <f t="shared" si="4"/>
+        <v>10560</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B38" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C38" s="22">
+        <v>7</v>
+      </c>
+      <c r="D38" s="2">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+      <c r="E38" s="2">
+        <f t="shared" si="4"/>
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B39" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C39" s="14">
+        <v>7</v>
+      </c>
+      <c r="D39" s="2">
+        <f>20</f>
+        <v>20</v>
+      </c>
+      <c r="E39" s="2">
+        <f t="shared" si="4"/>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B40" s="2"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="2">
-        <f>SUM(E6:E34)</f>
-        <v>2584.5</v>
+      <c r="E40" s="2">
+        <f>SUM(E6:E39)</f>
+        <v>30497</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B24:C24"/>
+  <mergeCells count="7">
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B23:C23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B3:I55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="5" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="42" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="34">
+        <v>1</v>
+      </c>
+      <c r="D5" s="34">
+        <v>220</v>
+      </c>
+      <c r="E5" s="43">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="32">
+        <v>1</v>
+      </c>
+      <c r="D6" s="32">
+        <v>52</v>
+      </c>
+      <c r="E6" s="45">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="44" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="32">
+        <v>2</v>
+      </c>
+      <c r="D7" s="32">
+        <v>4</v>
+      </c>
+      <c r="E7" s="45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="32">
+        <v>4</v>
+      </c>
+      <c r="D8" s="32">
+        <v>2</v>
+      </c>
+      <c r="E8" s="45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="32">
+        <v>2</v>
+      </c>
+      <c r="D9" s="32">
+        <v>3</v>
+      </c>
+      <c r="E9" s="45">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="32">
+        <v>2</v>
+      </c>
+      <c r="D10" s="32">
+        <v>2</v>
+      </c>
+      <c r="E10" s="45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="32">
+        <v>4</v>
+      </c>
+      <c r="D11" s="32">
+        <v>1</v>
+      </c>
+      <c r="E11" s="45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="44" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="32">
+        <v>8</v>
+      </c>
+      <c r="D12" s="32">
+        <v>1</v>
+      </c>
+      <c r="E12" s="45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="32">
+        <v>2</v>
+      </c>
+      <c r="D13" s="32">
+        <v>2</v>
+      </c>
+      <c r="E13" s="45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="32">
+        <v>5</v>
+      </c>
+      <c r="E14" s="45">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="44" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="32">
+        <v>10</v>
+      </c>
+      <c r="E15" s="45">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="39">
+        <v>5</v>
+      </c>
+      <c r="D16" s="39">
+        <v>5</v>
+      </c>
+      <c r="E16" s="47">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="49" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="42" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="34">
+        <v>2</v>
+      </c>
+      <c r="D20" s="34">
+        <v>25</v>
+      </c>
+      <c r="E20" s="43">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B21" s="44" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="32">
+        <v>1</v>
+      </c>
+      <c r="D21" s="32">
+        <v>20</v>
+      </c>
+      <c r="E21" s="45">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="46" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="39">
+        <v>2</v>
+      </c>
+      <c r="D22" s="39">
+        <v>5</v>
+      </c>
+      <c r="E22" s="47">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="34">
+        <v>223</v>
+      </c>
+      <c r="E26" s="43">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="32">
+        <v>12</v>
+      </c>
+      <c r="E27" s="45">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="32">
+        <v>1</v>
+      </c>
+      <c r="D28" s="32">
+        <v>60</v>
+      </c>
+      <c r="E28" s="45">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="32">
+        <v>1</v>
+      </c>
+      <c r="D29" s="32">
+        <v>60</v>
+      </c>
+      <c r="E29" s="45">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="32">
+        <v>20</v>
+      </c>
+      <c r="E30" s="45">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="44" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="32">
+        <v>2</v>
+      </c>
+      <c r="D31" s="32">
+        <v>2</v>
+      </c>
+      <c r="E31" s="45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" s="39">
+        <v>1</v>
+      </c>
+      <c r="D32" s="39">
+        <v>45</v>
+      </c>
+      <c r="E32" s="47">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="37" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="D36" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="51">
+        <v>1</v>
+      </c>
+      <c r="D37" s="51">
+        <v>150</v>
+      </c>
+      <c r="E37" s="52">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="34">
+        <v>240</v>
+      </c>
+      <c r="E41" s="43">
+        <v>4320</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B42" s="44" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="D42" s="32">
+        <v>240</v>
+      </c>
+      <c r="E42" s="45">
+        <v>8160</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="44" t="s">
+        <v>110</v>
+      </c>
+      <c r="C43" s="32" t="s">
+        <v>111</v>
+      </c>
+      <c r="D43" s="32">
+        <v>240</v>
+      </c>
+      <c r="E43" s="45">
+        <v>2880</v>
+      </c>
+      <c r="I43">
+        <f>SUM(C50:C54)</f>
+        <v>30437</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="C44" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D44" s="32">
+        <v>240</v>
+      </c>
+      <c r="E44" s="45">
+        <v>10560</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="C45" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="D45" s="32">
+        <v>240</v>
+      </c>
+      <c r="E45" s="45">
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="46" t="s">
+        <v>116</v>
+      </c>
+      <c r="C46" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="D46" s="39">
+        <v>20</v>
+      </c>
+      <c r="E46" s="47">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="40" t="s">
+        <v>117</v>
+      </c>
+      <c r="C47" s="41"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="37" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="49" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C49" s="37" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="C50" s="34">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C51" s="32">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B52" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C52" s="32">
+        <v>2158</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C53" s="32">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="54" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="C54" s="39">
+        <v>27680</v>
+      </c>
+    </row>
+    <row r="55" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="C55" s="37" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>